<commit_message>
Recapture v7 multi-line baselines after shared-market investment fix
WC-only baseline byte-identical (unchanged). WC+GL and WC+GL+PR updated:
GL and Property investment income shifts now that all lines share the same
per-year asset-class market draws instead of independent per-line streams.
Underwriting (premium, loss ratio) unchanged; only investment income and the
surplus it feeds moved. Determinism double-export verified byte-identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KByPnmZqFHAjC6MDpsfvdF
</commit_message>
<xml_diff>
--- a/baselines/BASELINE_v7_WC_GL.xlsx
+++ b/baselines/BASELINE_v7_WC_GL.xlsx
@@ -1225,13 +1225,13 @@
         <v>Invested Assets</v>
       </c>
       <c r="C49">
-        <v>37138809</v>
+        <v>36854117</v>
       </c>
       <c r="D49">
-        <v>42235889</v>
+        <v>41928179</v>
       </c>
       <c r="E49">
-        <v>47546892</v>
+        <v>46440777</v>
       </c>
     </row>
     <row r="50">
@@ -1242,13 +1242,13 @@
         <v>Investment Return Rate</v>
       </c>
       <c r="C50">
-        <v>0.030237033662821607</v>
+        <v>0.02984604461187138</v>
       </c>
       <c r="D50">
-        <v>0.045381663442640656</v>
+        <v>0.02667249985579053</v>
       </c>
       <c r="E50">
-        <v>0.038318292211466695</v>
+        <v>0.027616823897519748</v>
       </c>
     </row>
     <row r="51">
@@ -1259,13 +1259,13 @@
         <v>Investment Income</v>
       </c>
       <c r="C51">
-        <v>1122967</v>
+        <v>1099950</v>
       </c>
       <c r="D51">
-        <v>1916735</v>
+        <v>1118329</v>
       </c>
       <c r="E51">
-        <v>1821916</v>
+        <v>1282547</v>
       </c>
     </row>
     <row r="52">
@@ -1276,13 +1276,13 @@
         <v>Net Income</v>
       </c>
       <c r="C52">
-        <v>1635586</v>
+        <v>1612568</v>
       </c>
       <c r="D52">
-        <v>2869671</v>
+        <v>2071265</v>
       </c>
       <c r="E52">
-        <v>8314094</v>
+        <v>7774725</v>
       </c>
     </row>
     <row r="53">
@@ -1497,13 +1497,13 @@
         <v>Beginning Investments</v>
       </c>
       <c r="C65">
-        <v>37138809</v>
+        <v>36854117</v>
       </c>
       <c r="D65">
-        <v>42235889</v>
+        <v>41928179</v>
       </c>
       <c r="E65">
-        <v>47546892</v>
+        <v>46440777</v>
       </c>
     </row>
     <row r="66">
@@ -1514,13 +1514,13 @@
         <v>Ending Investments</v>
       </c>
       <c r="C66">
-        <v>42235889</v>
+        <v>41928179</v>
       </c>
       <c r="D66">
-        <v>47546892</v>
+        <v>46440777</v>
       </c>
       <c r="E66">
-        <v>54433062</v>
+        <v>52787578</v>
       </c>
     </row>
     <row r="67">
@@ -1548,13 +1548,13 @@
         <v>Total Assets</v>
       </c>
       <c r="C68">
-        <v>47630549</v>
+        <v>47322839</v>
       </c>
       <c r="D68">
-        <v>52901653</v>
+        <v>51795538</v>
       </c>
       <c r="E68">
-        <v>59470138</v>
+        <v>57824654</v>
       </c>
     </row>
     <row r="69">
@@ -1616,13 +1616,13 @@
         <v>Beginning Surplus</v>
       </c>
       <c r="C72">
-        <v>25002661</v>
+        <v>24717969</v>
       </c>
       <c r="D72">
-        <v>26638247</v>
+        <v>26330537</v>
       </c>
       <c r="E72">
-        <v>29507917</v>
+        <v>28401802</v>
       </c>
     </row>
     <row r="73">
@@ -1633,13 +1633,13 @@
         <v>Surplus from Income</v>
       </c>
       <c r="C73">
-        <v>26638247</v>
+        <v>26330537</v>
       </c>
       <c r="D73">
-        <v>29507917</v>
+        <v>28401802</v>
       </c>
       <c r="E73">
-        <v>37822011</v>
+        <v>36176527</v>
       </c>
     </row>
     <row r="74">
@@ -1650,13 +1650,13 @@
         <v>Ending Surplus</v>
       </c>
       <c r="C74">
-        <v>26638247</v>
+        <v>26330537</v>
       </c>
       <c r="D74">
-        <v>29507917</v>
+        <v>28401802</v>
       </c>
       <c r="E74">
-        <v>37822011</v>
+        <v>36176527</v>
       </c>
     </row>
     <row r="75">
@@ -1854,13 +1854,13 @@
         <v>Surplus</v>
       </c>
       <c r="C86">
-        <v>26638247</v>
+        <v>26330537</v>
       </c>
       <c r="D86">
-        <v>29507917</v>
+        <v>28401802</v>
       </c>
       <c r="E86">
-        <v>37822011</v>
+        <v>36176527</v>
       </c>
     </row>
     <row r="87">
@@ -1871,13 +1871,13 @@
         <v>Excess Available Surplus</v>
       </c>
       <c r="C87">
-        <v>8842419</v>
+        <v>8534709</v>
       </c>
       <c r="D87">
-        <v>9183019</v>
+        <v>8076904</v>
       </c>
       <c r="E87">
-        <v>18753732</v>
+        <v>17108247</v>
       </c>
     </row>
     <row r="88">
@@ -1888,13 +1888,13 @@
         <v>Excess Capital Ratio</v>
       </c>
       <c r="C88">
-        <v>0.49688155712324966</v>
+        <v>0.47959044685257235</v>
       </c>
       <c r="D88">
-        <v>0.45181133621270675</v>
+        <v>0.3973896532075068</v>
       </c>
       <c r="E88">
-        <v>0.9835041040774051</v>
+        <v>0.897209791482031</v>
       </c>
     </row>
     <row r="89">
@@ -3381,10 +3381,10 @@
         <v>1.3109577750035035</v>
       </c>
       <c r="D86">
-        <v>0.9955385830764771</v>
+        <v>0.9955385830764767</v>
       </c>
       <c r="E86">
-        <v>1.0995651883422943</v>
+        <v>1.0995651883422939</v>
       </c>
     </row>
     <row r="87">
@@ -4205,13 +4205,13 @@
         <v>Invested Assets</v>
       </c>
       <c r="C47">
-        <v>16353214</v>
+        <v>16068522</v>
       </c>
       <c r="D47">
-        <v>18361880</v>
+        <v>18054170</v>
       </c>
       <c r="E47">
-        <v>21208230</v>
+        <v>20102115</v>
       </c>
     </row>
     <row r="48">
@@ -4222,13 +4222,13 @@
         <v>Investment Return Rate</v>
       </c>
       <c r="C48">
-        <v>0.030733996516013377</v>
+        <v>0.029846044611871386</v>
       </c>
       <c r="D48">
-        <v>0.06970720915315894</v>
+        <v>0.02667249985579053</v>
       </c>
       <c r="E48">
-        <v>0.051608526746957165</v>
+        <v>0.027616823897519745</v>
       </c>
     </row>
     <row r="49">
@@ -4239,13 +4239,13 @@
         <v>Investment Income</v>
       </c>
       <c r="C49">
-        <v>502600</v>
+        <v>479582</v>
       </c>
       <c r="D49">
-        <v>1279955</v>
+        <v>481550</v>
       </c>
       <c r="E49">
-        <v>1094526</v>
+        <v>555157</v>
       </c>
     </row>
     <row r="50">
@@ -4256,13 +4256,13 @@
         <v>Net Income</v>
       </c>
       <c r="C50">
-        <v>-95762</v>
+        <v>-118780</v>
       </c>
       <c r="D50">
-        <v>2016686</v>
+        <v>1218281</v>
       </c>
       <c r="E50">
-        <v>6282500</v>
+        <v>5743131</v>
       </c>
     </row>
     <row r="51">
@@ -4477,13 +4477,13 @@
         <v>Beginning Investments</v>
       </c>
       <c r="C63">
-        <v>16353214</v>
+        <v>16068522</v>
       </c>
       <c r="D63">
-        <v>18361880</v>
+        <v>18054170</v>
       </c>
       <c r="E63">
-        <v>21208230</v>
+        <v>20102115</v>
       </c>
     </row>
     <row r="64">
@@ -4494,13 +4494,13 @@
         <v>Ending Investments</v>
       </c>
       <c r="C64">
-        <v>18361880</v>
+        <v>18054170</v>
       </c>
       <c r="D64">
-        <v>21208230</v>
+        <v>20102115</v>
       </c>
       <c r="E64">
-        <v>25560697</v>
+        <v>23915213</v>
       </c>
     </row>
     <row r="65">
@@ -4528,13 +4528,13 @@
         <v>Total Assets</v>
       </c>
       <c r="C66">
-        <v>21804050</v>
+        <v>21496341</v>
       </c>
       <c r="D66">
-        <v>24283995</v>
+        <v>23177880</v>
       </c>
       <c r="E66">
-        <v>28428578</v>
+        <v>26783094</v>
       </c>
     </row>
     <row r="67">
@@ -4596,13 +4596,13 @@
         <v>Beginning Surplus</v>
       </c>
       <c r="C70">
-        <v>9310013</v>
+        <v>9025321</v>
       </c>
       <c r="D70">
-        <v>9214250</v>
+        <v>8906541</v>
       </c>
       <c r="E70">
-        <v>11230937</v>
+        <v>10124821</v>
       </c>
     </row>
     <row r="71">
@@ -4613,13 +4613,13 @@
         <v>Surplus from Income</v>
       </c>
       <c r="C71">
-        <v>9214250</v>
+        <v>8906541</v>
       </c>
       <c r="D71">
-        <v>11230937</v>
+        <v>10124821</v>
       </c>
       <c r="E71">
-        <v>17513437</v>
+        <v>15867953</v>
       </c>
     </row>
     <row r="72">
@@ -4630,13 +4630,13 @@
         <v>Ending Surplus</v>
       </c>
       <c r="C72">
-        <v>9214250</v>
+        <v>8906541</v>
       </c>
       <c r="D72">
-        <v>11230937</v>
+        <v>10124821</v>
       </c>
       <c r="E72">
-        <v>17513437</v>
+        <v>15867953</v>
       </c>
     </row>
     <row r="73">
@@ -4834,13 +4834,13 @@
         <v>Surplus</v>
       </c>
       <c r="C84">
-        <v>9214250</v>
+        <v>8906541</v>
       </c>
       <c r="D84">
-        <v>11230937</v>
+        <v>10124821</v>
       </c>
       <c r="E84">
-        <v>17513437</v>
+        <v>15867953</v>
       </c>
     </row>
     <row r="85">
@@ -4851,13 +4851,13 @@
         <v>Excess Available Surplus</v>
       </c>
       <c r="C85">
-        <v>-1041848</v>
+        <v>-1349558</v>
       </c>
       <c r="D85">
-        <v>64960</v>
+        <v>-1041155</v>
       </c>
       <c r="E85">
-        <v>8117909</v>
+        <v>6472425</v>
       </c>
     </row>
     <row r="86">
@@ -4868,13 +4868,13 @@
         <v>Excess Capital Ratio</v>
       </c>
       <c r="C86">
-        <v>-0.10158327615482862</v>
+        <v>-0.1315858760846424</v>
       </c>
       <c r="D86">
-        <v>0.005817660096269805</v>
+        <v>-0.09324354870781587</v>
       </c>
       <c r="E86">
-        <v>0.8640185095407007</v>
+        <v>0.6888836755000718</v>
       </c>
     </row>
     <row r="87">
@@ -4888,7 +4888,7 @@
         <v>Deficient</v>
       </c>
       <c r="D87" t="str">
-        <v>Adequate</v>
+        <v>Thin</v>
       </c>
       <c r="E87" t="str">
         <v>Strong</v>

</xml_diff>